<commit_message>
fix(analytics): optimizar query de churn general para resumen consolidado
</commit_message>
<xml_diff>
--- a/data/processed/reporte_ejecutivo_churn.xlsx
+++ b/data/processed/reporte_ejecutivo_churn.xlsx
@@ -415,49 +415,34 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Churn</t>
+          <t>total_clientes</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>total_clientes</t>
+          <t>clientes_perdidos</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>porcentaje</t>
+          <t>churn_rate_global</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
+      <c r="A2" t="n">
+        <v>7043</v>
       </c>
       <c r="B2" t="n">
-        <v>5174</v>
+        <v>1869</v>
       </c>
       <c r="C2" t="n">
-        <v>73.45999999999999</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>1869</v>
-      </c>
-      <c r="C3" t="n">
         <v>26.54</v>
       </c>
     </row>

</xml_diff>